<commit_message>
08.03.2026 -Edit Old Symbol and Footprint -Add izm5.174.020 -Add pogopin p75-b1 -Add Solder Jumper -Add Fiducal Footprint
</commit_message>
<xml_diff>
--- a/Database_Lib.xlsx
+++ b/Database_Lib.xlsx
@@ -8,16 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\altium\Altium_Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA2EB328-8712-4870-8508-9B57F4496228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A755750-FF16-4A37-8779-0E3068644DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4968" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Resistor" sheetId="1" r:id="rId1"/>
+    <sheet name="Resistor" sheetId="3" r:id="rId1"/>
+    <sheet name="Capacitor" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Resistor!$A$1:$I$1</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="31">
   <si>
     <t>GOST_VALUE</t>
   </si>
@@ -97,6 +95,42 @@
   </si>
   <si>
     <t>RC0402FR-070RL</t>
+  </si>
+  <si>
+    <t>50В</t>
+  </si>
+  <si>
+    <t>0,1 мкФ</t>
+  </si>
+  <si>
+    <t>С0603</t>
+  </si>
+  <si>
+    <t>0.1uF</t>
+  </si>
+  <si>
+    <t>10%</t>
+  </si>
+  <si>
+    <t>GOST_TKE</t>
+  </si>
+  <si>
+    <t>X7R</t>
+  </si>
+  <si>
+    <t>CC0603KRX7R9BB104</t>
+  </si>
+  <si>
+    <t>Capacitor</t>
+  </si>
+  <si>
+    <t>5.1 кОм</t>
+  </si>
+  <si>
+    <t>5.1k</t>
+  </si>
+  <si>
+    <t>RC0603FR-075K1L</t>
   </si>
 </sst>
 </file>
@@ -429,19 +463,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06DB4D5C-124F-40F8-A1BC-9516EF6D22C9}">
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.21875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="30.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -533,13 +567,128 @@
         <v>Resistor 0603 (1608) 0.1 Вт 0 Ом 1%</v>
       </c>
     </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" t="str">
+        <f>F4 &amp;" "&amp;B4&amp;" "&amp;C4&amp;" "&amp;D4&amp;" "&amp;E4</f>
+        <v>Resistor 0603 (1608) 0.1 Вт 5.1 кОм 1%</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I3">
-      <sortCondition ref="D1"/>
-    </sortState>
-  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I3">
+    <sortCondition ref="D2:D3"/>
+  </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62FED977-E1E5-4AD4-AEED-B08864737075}">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="34" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" t="str">
+        <f>G2 &amp;" "&amp;B2&amp;" "&amp;C2&amp;" "&amp;D2&amp;" "&amp;E2</f>
+        <v>Capacitor 0402 (1005) 50В 0,1 мкФ 10%</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>